<commit_message>
Mejoras agregadas: Seleccionar area, exporta a word, bd con proyeccion a docker
</commit_message>
<xml_diff>
--- a/intake/intake_informes.xlsx
+++ b/intake/intake_informes.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tramites" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo_Equipos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Responsables" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1094,4 +1095,115 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>etiqueta_responsable</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>nombre_responsable</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Farmacia Corporativa</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>JEFE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ALEJANDRO IZQUIERDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Contabilidad</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A CARGO</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ROBERTO DIAZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sistemas</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>JEFATURA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>STEFAN MANDUJANO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CSO</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>JEFE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GIANNINA DOMINGUEZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Nota: al elegir un area en el wizard, se sugiere automaticamente el responsable de esta tabla (editable en el momento). Si el area no esta aqui, el wizard pide los datos a mano.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>